<commit_message>
Actualización automática 2026-05-18 12:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
+++ b/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
@@ -435,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -512,19 +512,46 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PYCCA S.A.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>107.16</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="3" t="n">
+        <v>107.16</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -539,11 +566,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
@@ -715,84 +742,144 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="Q3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
-        </is>
-      </c>
-      <c r="R3" s="4" t="inlineStr">
-        <is>
-          <t>0 de 1</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PYCCA S.A.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>0 de 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-05-22 12:30:22
</commit_message>
<xml_diff>
--- a/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
+++ b/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
@@ -448,7 +448,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -564,7 +564,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>80</v>
+        <v>720.05</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0</v>
@@ -581,7 +581,7 @@
         <v>58.9</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>80</v>
+        <v>720.05</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>0</v>
@@ -875,7 +875,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>80</v>
+        <v>720.05</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -992,9 +992,9 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1068,13 +1068,13 @@
         <v>15000</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>80</v>
+        <v>720.05</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>14920</v>
+        <v>14279.95</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.005333333333333333</v>
+        <v>0.04800333333333333</v>
       </c>
     </row>
     <row r="4">
@@ -1087,13 +1087,13 @@
         <v>15000</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>80</v>
+        <v>720.05</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>14920</v>
+        <v>14279.95</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.005333333333333333</v>
+        <v>0.04800333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-02 10:30:21
</commit_message>
<xml_diff>
--- a/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
+++ b/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -510,7 +510,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>503.56</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0</v>
@@ -581,7 +581,7 @@
         <v>720.05</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0</v>
+        <v>503.56</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>0</v>
@@ -728,7 +728,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>503.56</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
@@ -901,7 +901,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>0 de 3</t>
+          <t>1 de 3</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática 2026-06-17 09:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
+++ b/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
@@ -591,7 +591,7 @@
         <v>720.05</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>200.02</v>
+        <v>392.56</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>0</v>
@@ -608,7 +608,7 @@
         <v>720.05</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>703.58</v>
+        <v>896.12</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -962,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>200.02</v>
+        <v>392.56</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -1155,13 +1155,13 @@
         <v>13101</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>200.02</v>
+        <v>392.56</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>12900.98</v>
+        <v>12708.44</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.01526753682924968</v>
+        <v>0.02996412487596367</v>
       </c>
     </row>
     <row r="4">
@@ -1174,13 +1174,13 @@
         <v>13101</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>703.58</v>
+        <v>896.12</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>12397.42</v>
+        <v>12204.88</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.05370429738187925</v>
+        <v>0.06840088542859324</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-26 09:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
+++ b/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
@@ -510,7 +510,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>320.79</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0</v>
@@ -662,7 +662,7 @@
         <v>720.05</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>896.12</v>
+        <v>1216.91</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>0</v>
@@ -836,7 +836,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>320.79</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>1 de 6</t>
+          <t>2 de 6</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
@@ -1329,13 +1329,13 @@
         <v>13101</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>392.56</v>
+        <v>713.35</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>12708.44</v>
+        <v>12387.65</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.02996412487596367</v>
+        <v>0.05445004198152813</v>
       </c>
     </row>
     <row r="4">
@@ -1348,13 +1348,13 @@
         <v>13101</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>896.12</v>
+        <v>1216.91</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>12204.88</v>
+        <v>11884.09</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.06840088542859324</v>
+        <v>0.09288680253415771</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-30 10:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
+++ b/data/CASTRO CALDERON VERONICA SOBEIDA.xlsx
@@ -440,12 +440,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -497,20 +497,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1125.31</v>
+        <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>24.18</v>
+        <v>0</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>320.79</v>
+        <v>503.56</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0</v>
@@ -524,7 +524,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>MEGAMETALES S.A.</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -537,7 +537,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>503.56</v>
+        <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0</v>
@@ -551,7 +551,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MEGAMETALES S.A.</t>
+          <t>MOBILTROICORP S.A.</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -578,14 +578,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MOBILTROICORP S.A.</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>58.9</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -605,66 +605,39 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>720.05</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>392.56</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3" t="n">
         <v>58.9</v>
       </c>
-      <c r="E6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>720.05</v>
       </c>
-      <c r="F7" s="2" t="n">
-        <v>392.56</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="C8" s="3" t="n">
-        <v>1125.31</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>83.08</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>720.05</v>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>1216.91</v>
-      </c>
-      <c r="G8" s="3" t="n">
+      <c r="F7" s="3" t="n">
+        <v>896.12</v>
+      </c>
+      <c r="G7" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -679,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -802,14 +775,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>503.56</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
@@ -836,7 +809,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>320.79</v>
+        <v>0</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -862,14 +835,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>MEGAMETALES S.A.</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>503.56</v>
+        <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
@@ -922,7 +895,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MEGAMETALES S.A.</t>
+          <t>MOBILTROICORP S.A.</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -982,7 +955,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MOBILTROICORP S.A.</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -1042,7 +1015,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -1076,7 +1049,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0</v>
+        <v>392.56</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
@@ -1095,144 +1068,84 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="2" t="n">
-        <v>392.56</v>
-      </c>
-      <c r="N7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>1 de 6</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>2 de 6</t>
-        </is>
-      </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="P8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="Q8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
-        </is>
-      </c>
-      <c r="R8" s="4" t="inlineStr">
-        <is>
-          <t>0 de 6</t>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1 de 5</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>1 de 5</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
+        </is>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>0 de 5</t>
         </is>
       </c>
     </row>

</xml_diff>